<commit_message>
Update Tagged 30 Accounts with refined selections and formatting
- Improved account selections with better revenue sorting
- Enhanced Excel formatting with blue headers and borders

https://claude.ai/code/session_018CdomwcM2t3v3UWZ6osXnY
</commit_message>
<xml_diff>
--- a/backend/analysis/Tagged_30_Accounts.xlsx
+++ b/backend/analysis/Tagged_30_Accounts.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,19 +26,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -82,14 +76,16 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,11 +455,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,7 +512,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>BHP GROUP LIMITED</t>
+          <t>AGL ENERGY LIMITED</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -529,12 +525,12 @@
           <t>LE - AU</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>N/A (Major mining company)</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>SAP Install Base account</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -542,7 +538,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>WOOLWORTHS GROUP LIMITED</t>
+          <t>AMCOR PLC</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -555,12 +551,12 @@
           <t>LE - AU</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>N/A (Major retailer)</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>SAP Install Base account</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -568,7 +564,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>COMMONWEALTH BANK OF AUSTRALIA</t>
+          <t>Ampol Australia Petroleum Pty Ltd</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -581,14 +577,10 @@
           <t>LE - AU</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>N/A (Major bank)</t>
-        </is>
-      </c>
+      <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Listed as 'Commonwealth Bank of Australia'</t>
+          <t>SAP Install Base account</t>
         </is>
       </c>
     </row>
@@ -613,10 +605,14 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>$433.5B turnover</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr"/>
+          <t>$433.5B</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Wholesale Distribution</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -639,10 +635,14 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>$244.3B turnover</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr"/>
+          <t>$244.3B</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Energy &amp; Utility</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -665,10 +665,14 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>$130.3B turnover</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
+          <t>$130.3B</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -691,7 +695,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>$103.5B revenue</t>
+          <t>$103.5B</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr"/>
@@ -717,7 +721,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>$24.7B revenue</t>
+          <t>$24.7B</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr"/>
@@ -743,7 +747,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>$22.8B revenue</t>
+          <t>$22.8B</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
@@ -754,7 +758,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Indonesia - Cargo Transportation &amp; Logistics (Fortune 500)</t>
+          <t>Cargo Transportation &amp; Logistics Service (INDONESIA)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -769,12 +773,12 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>$129.7B turnover</t>
+          <t>$129.7B</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Industry: Cargo Transportation &amp; Logistics Service, Fortune global 500</t>
+          <t>Fortune global 500</t>
         </is>
       </c>
     </row>
@@ -784,7 +788,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Indonesia - Energy Company (Fortune 500)</t>
+          <t>Information Technology (Ireland)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -799,12 +803,12 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>$64.9B turnover</t>
+          <t>$64.9B</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Industry: Information Technology, Fortune global 500</t>
+          <t>Fortune global 500</t>
         </is>
       </c>
     </row>
@@ -827,12 +831,12 @@
           <t>LE - TH</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Banking &amp; Financial Services</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -853,12 +857,12 @@
           <t>LE - TH</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Oil and Gas</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -881,10 +885,14 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>$68.8B group revenue</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr"/>
+          <t>$68.8B</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -907,10 +915,14 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>$68.8B group revenue</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr"/>
+          <t>$68.8B</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -930,12 +942,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Genting Admin Services Sdn Bhd</t>
+          <t>Prime Minister's Office</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>MY</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -950,7 +962,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>2024 MA Fees rank: 465</t>
+          <t>Public Sector</t>
         </is>
       </c>
     </row>
@@ -960,12 +972,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Social Security System</t>
+          <t>Provincial Electricity Authority</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>ICN</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -980,7 +992,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>2024 MA Fees rank: 464</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
@@ -990,12 +1002,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Lembaga Penjamin Simpanan</t>
+          <t>Ministry of Defence C/O</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -1010,7 +1022,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>2024 MA Fees rank: 462</t>
+          <t>Defense and Security</t>
         </is>
       </c>
     </row>
@@ -1020,12 +1032,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Emperador Distillers Inc.</t>
+          <t>Jabatan Akauntan Negara Malaysia</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>MY</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1040,7 +1052,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>2024 MA Fees rank: 461</t>
+          <t>Public Sector</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1062,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Boustead Petroleum Marketing Sdn Bhd</t>
+          <t>Kementerian Kewangan Malaysia</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1070,7 +1082,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>2024 MA Fees rank: 460</t>
+          <t>Public Sector</t>
         </is>
       </c>
     </row>
@@ -1107,10 +1119,14 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>180 MB (ERP)</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr"/>
+          <t>ERP MB: 180.0</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Cloud: No</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -1133,10 +1149,14 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>175 MB (ERP)</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr"/>
+          <t>ERP MB: 175.0</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Cloud: No</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -1159,10 +1179,14 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>157 MB (ERP)</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr"/>
+          <t>ERP MB: 157.0</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Cloud: No</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -1185,10 +1209,14 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>126 MB (ERP)</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr"/>
+          <t>ERP MB: 126.0</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Cloud: No</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -1211,10 +1239,14 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>117 MB (ERP)</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr"/>
+          <t>ERP MB: 117.0</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Cloud: No</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -1222,7 +1254,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Panasonic Life Solutions India Priv</t>
+          <t>Plasser India Pvt. Limited</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -1232,15 +1264,19 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>AMS Inactive</t>
+          <t>AMS Active</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>$840 contract value</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr"/>
+          <t>ERP MB: 89.0</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Cloud: No</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -1248,12 +1284,12 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Thaicom Public Company Limited</t>
+          <t>Sms India Private Limited</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
@@ -1263,10 +1299,14 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>$840 contract value</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr"/>
+          <t>AMS CV: 9.800.000</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Not Active SAP Customer</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -1274,7 +1314,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Suven Pharmaceuticals Limited</t>
+          <t>KIMS Health Care Management Limited</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -1289,10 +1329,14 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>$750 contract value</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr"/>
+          <t>AMS CV: 6.319.100</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Not Active SAP Customer</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -1300,12 +1344,12 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Eastern Water Resources Development</t>
+          <t>Kluber Lubrication India Private Lt</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -1315,10 +1359,14 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>$750 contract value</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr"/>
+          <t>AMS CV: 5.691.600</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Not Active SAP Customer</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -1326,7 +1374,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Nippon Paint Lanka (Private) Limite</t>
+          <t>SPI TECHNOLOGIES INDIA PVT LTD</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -1341,10 +1389,14 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>$702 contract value</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr"/>
+          <t>AMS CV: 2.530.000</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Not Active SAP Customer</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>